<commit_message>
data_juste modéle a modifier encore quelque erreurs
</commit_message>
<xml_diff>
--- a/ARG_WB_timeseries.xlsx
+++ b/ARG_WB_timeseries.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Control of Corruption</t>
   </si>
@@ -35,6 +35,9 @@
   </si>
   <si>
     <t>Foreign direct investment, net outflows (BoP, current US$)</t>
+  </si>
+  <si>
+    <t>GDP (current US$)</t>
   </si>
   <si>
     <t>GDP growth (annual %)</t>
@@ -443,12 +446,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X36"/>
+  <dimension ref="A1:Y36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:24">
+    <row r="1" spans="1:25">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -519,8 +522,11 @@
       <c r="X1" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:24">
+      <c r="Y1" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25">
       <c r="A2" s="1">
         <v>1990</v>
       </c>
@@ -543,43 +549,46 @@
         <v>34902990</v>
       </c>
       <c r="I2">
+        <v>141352654305.163</v>
+      </c>
+      <c r="J2">
         <v>-2.46721377810472</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>4315.33403111588</v>
       </c>
-      <c r="L2">
+      <c r="M2">
         <v>3.13542839161188</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>10.3254404487432</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>10.3875396339054</v>
       </c>
-      <c r="O2">
+      <c r="P2">
         <v>4.63132240741775</v>
       </c>
-      <c r="Q2">
+      <c r="R2">
         <v>8.65453523501721</v>
       </c>
-      <c r="R2">
+      <c r="S2">
         <v>-0.107803024709003</v>
       </c>
-      <c r="T2">
+      <c r="U2">
         <v>4.83851314669697</v>
       </c>
-      <c r="U2">
+      <c r="V2">
         <v>6222040362.99099</v>
       </c>
-      <c r="V2">
+      <c r="W2">
         <v>5.69957895846503</v>
       </c>
-      <c r="W2">
+      <c r="X2">
         <v>14.9908589999441</v>
       </c>
     </row>
-    <row r="3" spans="1:24">
+    <row r="3" spans="1:25">
       <c r="A3" s="1">
         <v>1991</v>
       </c>
@@ -602,49 +611,52 @@
         <v>49385690</v>
       </c>
       <c r="I3">
+        <v>189719984268.485</v>
+      </c>
+      <c r="J3">
         <v>9.133110567389609</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>5709.24784079504</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>46.8</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>3.32176128752774</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>11.2055409345172</v>
       </c>
-      <c r="N3">
+      <c r="O3">
         <v>11.1620910357746</v>
       </c>
-      <c r="O3">
+      <c r="P3">
         <v>6.07801081056698</v>
       </c>
-      <c r="Q3">
+      <c r="R3">
         <v>11.0514735626967</v>
       </c>
-      <c r="R3">
+      <c r="S3">
         <v>-0.229466322749109</v>
       </c>
-      <c r="T3">
+      <c r="U3">
         <v>5.00823654744009</v>
       </c>
-      <c r="U3">
+      <c r="V3">
         <v>7462543636.08691</v>
       </c>
-      <c r="V3">
+      <c r="W3">
         <v>5.09620553340786</v>
       </c>
-      <c r="W3">
+      <c r="X3">
         <v>13.7530541588891</v>
       </c>
-      <c r="X3">
+      <c r="Y3">
         <v>5.44</v>
       </c>
     </row>
-    <row r="4" spans="1:24">
+    <row r="4" spans="1:25">
       <c r="A4" s="1">
         <v>1992</v>
       </c>
@@ -667,49 +679,52 @@
         <v>1165914300</v>
       </c>
       <c r="I4">
+        <v>228778917308.17</v>
+      </c>
+      <c r="J4">
         <v>7.93729155643076</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>6789.99611136495</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>45.5</v>
       </c>
-      <c r="L4">
+      <c r="M4">
         <v>2.97553802761558</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>11.8011099217048</v>
       </c>
-      <c r="N4">
+      <c r="O4">
         <v>12.2806411476509</v>
       </c>
-      <c r="O4">
+      <c r="P4">
         <v>8.132793114315639</v>
       </c>
-      <c r="Q4">
+      <c r="R4">
         <v>9.80266060465569</v>
       </c>
-      <c r="R4">
+      <c r="S4">
         <v>0.264562866283836</v>
       </c>
-      <c r="T4">
+      <c r="U4">
         <v>5.54792213441138</v>
       </c>
-      <c r="U4">
+      <c r="V4">
         <v>11447031156.7334</v>
       </c>
-      <c r="V4">
+      <c r="W4">
         <v>5.70506107278321</v>
       </c>
-      <c r="W4">
+      <c r="X4">
         <v>14.730980586353</v>
       </c>
-      <c r="X4">
+      <c r="Y4">
         <v>6.36</v>
       </c>
     </row>
-    <row r="5" spans="1:24">
+    <row r="5" spans="1:25">
       <c r="A5" s="1">
         <v>1993</v>
       </c>
@@ -732,49 +747,52 @@
         <v>705070000</v>
       </c>
       <c r="I5">
+        <v>236741715015.015</v>
+      </c>
+      <c r="J5">
         <v>8.206979072212279</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>6931.85596375876</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>44.8</v>
       </c>
-      <c r="L5">
+      <c r="M5">
         <v>13.5103784728742</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>14.2818561185834</v>
       </c>
-      <c r="N5">
+      <c r="O5">
         <v>15.0995556252854</v>
       </c>
-      <c r="O5">
+      <c r="P5">
         <v>9.313799914075631</v>
       </c>
-      <c r="Q5">
+      <c r="R5">
         <v>7.60836419725674</v>
       </c>
-      <c r="R5">
+      <c r="S5">
         <v>0.483203369491258</v>
       </c>
-      <c r="T5">
+      <c r="U5">
         <v>8.01513800555669</v>
       </c>
-      <c r="U5">
+      <c r="V5">
         <v>15499431243.972</v>
       </c>
-      <c r="V5">
+      <c r="W5">
         <v>6.74386056512176</v>
       </c>
-      <c r="W5">
+      <c r="X5">
         <v>16.223151447784</v>
       </c>
-      <c r="X5">
+      <c r="Y5">
         <v>10.1</v>
       </c>
     </row>
-    <row r="6" spans="1:24">
+    <row r="6" spans="1:25">
       <c r="A6" s="1">
         <v>1994</v>
       </c>
@@ -797,49 +815,52 @@
         <v>1012844000</v>
       </c>
       <c r="I6">
+        <v>257440000000</v>
+      </c>
+      <c r="J6">
         <v>5.83620070368526</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>7437.56242327594</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>45.9</v>
       </c>
-      <c r="L6">
+      <c r="M6">
         <v>13.1869043660659</v>
       </c>
-      <c r="M6">
+      <c r="N6">
         <v>14.9007924176507</v>
       </c>
-      <c r="N6">
+      <c r="O6">
         <v>14.8638517712865</v>
       </c>
-      <c r="O6">
+      <c r="P6">
         <v>10.6043971410814</v>
       </c>
-      <c r="Q6">
+      <c r="R6">
         <v>8.321037731422351</v>
       </c>
-      <c r="R6">
+      <c r="S6">
         <v>-0.32605655686762</v>
       </c>
-      <c r="T6">
+      <c r="U6">
         <v>8.12643722809198</v>
       </c>
-      <c r="U6">
+      <c r="V6">
         <v>16003265688.189</v>
       </c>
-      <c r="V6">
+      <c r="W6">
         <v>5.59678188654751</v>
       </c>
-      <c r="W6">
+      <c r="X6">
         <v>18.1343458669981</v>
       </c>
-      <c r="X6">
+      <c r="Y6">
         <v>11.76</v>
       </c>
     </row>
-    <row r="7" spans="1:24">
+    <row r="7" spans="1:25">
       <c r="A7" s="1">
         <v>1995</v>
       </c>
@@ -862,49 +883,52 @@
         <v>1497149000</v>
       </c>
       <c r="I7">
+        <v>258031750000</v>
+      </c>
+      <c r="J7">
         <v>-2.84520961057079</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>7357.6162773788</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>48.9</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <v>13.3494556774505</v>
       </c>
-      <c r="M7">
+      <c r="N7">
         <v>15.5112306915719</v>
       </c>
-      <c r="N7">
+      <c r="O7">
         <v>14.0262971514164</v>
       </c>
-      <c r="O7">
+      <c r="P7">
         <v>10.0910128307854</v>
       </c>
-      <c r="Q7">
+      <c r="R7">
         <v>10.2016545114294</v>
       </c>
-      <c r="R7">
+      <c r="S7">
         <v>-1.71796687810705</v>
       </c>
-      <c r="T7">
+      <c r="U7">
         <v>8.054357651723089</v>
       </c>
-      <c r="U7">
+      <c r="V7">
         <v>15979453701.6387</v>
       </c>
-      <c r="V7">
+      <c r="W7">
         <v>5.47248285450445</v>
       </c>
-      <c r="W7">
+      <c r="X7">
         <v>19.7714230903755</v>
       </c>
-      <c r="X7">
+      <c r="Y7">
         <v>18.8</v>
       </c>
     </row>
-    <row r="8" spans="1:24">
+    <row r="8" spans="1:25">
       <c r="A8" s="1">
         <v>1996</v>
       </c>
@@ -930,52 +954,55 @@
         <v>1600749000</v>
       </c>
       <c r="I8">
+        <v>272149750000</v>
+      </c>
+      <c r="J8">
         <v>5.52668982715234</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>7663.21271287469</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>49.5</v>
       </c>
-      <c r="L8">
+      <c r="M8">
         <v>12.5016776609201</v>
       </c>
-      <c r="M8">
+      <c r="N8">
         <v>15.1655476442657</v>
       </c>
-      <c r="N8">
+      <c r="O8">
         <v>13.0408350549651</v>
       </c>
-      <c r="O8">
+      <c r="P8">
         <v>11.0778716497076</v>
       </c>
-      <c r="Q8">
+      <c r="R8">
         <v>11.2133840525283</v>
       </c>
-      <c r="R8">
+      <c r="S8">
         <v>-2.33400912549065</v>
       </c>
-      <c r="S8">
+      <c r="T8">
         <v>0.111376881599426</v>
       </c>
-      <c r="T8">
+      <c r="U8">
         <v>8.17178777492906</v>
       </c>
-      <c r="U8">
+      <c r="V8">
         <v>19719017351.0624</v>
       </c>
-      <c r="V8">
+      <c r="W8">
         <v>5.89789511152116</v>
       </c>
-      <c r="W8">
+      <c r="X8">
         <v>21.5064684057215</v>
       </c>
-      <c r="X8">
+      <c r="Y8">
         <v>17.11</v>
       </c>
     </row>
-    <row r="9" spans="1:24">
+    <row r="9" spans="1:25">
       <c r="A9" s="1">
         <v>1997</v>
       </c>
@@ -998,49 +1025,52 @@
         <v>3652818000</v>
       </c>
       <c r="I9">
+        <v>292859000000</v>
+      </c>
+      <c r="J9">
         <v>8.1110467707457</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>8146.78710021431</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>49.1</v>
       </c>
-      <c r="L9">
+      <c r="M9">
         <v>12.0620142457633</v>
       </c>
-      <c r="M9">
+      <c r="N9">
         <v>15.0142218610321</v>
       </c>
-      <c r="N9">
+      <c r="O9">
         <v>13.6002991200544</v>
       </c>
-      <c r="O9">
+      <c r="P9">
         <v>12.7753287418177</v>
       </c>
-      <c r="Q9">
+      <c r="R9">
         <v>13.0351030804744</v>
       </c>
-      <c r="R9">
+      <c r="S9">
         <v>-1.65752119620705</v>
       </c>
-      <c r="T9">
+      <c r="U9">
         <v>8.690086355549941</v>
       </c>
-      <c r="U9">
+      <c r="V9">
         <v>22424600096.7817</v>
       </c>
-      <c r="V9">
+      <c r="W9">
         <v>5.47566058156948</v>
       </c>
-      <c r="W9">
+      <c r="X9">
         <v>23.3361788437439</v>
       </c>
-      <c r="X9">
+      <c r="Y9">
         <v>14.82</v>
       </c>
     </row>
-    <row r="10" spans="1:24">
+    <row r="10" spans="1:25">
       <c r="A10" s="1">
         <v>1998</v>
       </c>
@@ -1066,52 +1096,55 @@
         <v>2325477000</v>
       </c>
       <c r="I10">
+        <v>298948250000</v>
+      </c>
+      <c r="J10">
         <v>3.85017885156228</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>8218.992127646819</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>50.7</v>
       </c>
-      <c r="L10">
+      <c r="M10">
         <v>12.4947749986829</v>
       </c>
-      <c r="M10">
+      <c r="N10">
         <v>15.0988005449104</v>
       </c>
-      <c r="N10">
+      <c r="O10">
         <v>13.7561266874785</v>
       </c>
-      <c r="O10">
+      <c r="P10">
         <v>12.934446011977</v>
       </c>
-      <c r="Q10">
+      <c r="R10">
         <v>14.7114600687675</v>
       </c>
-      <c r="R10">
+      <c r="S10">
         <v>-1.58616081545886</v>
       </c>
-      <c r="S10">
+      <c r="T10">
         <v>-0.134649589657784</v>
       </c>
-      <c r="T10">
+      <c r="U10">
         <v>9.03052618638845</v>
       </c>
-      <c r="U10">
+      <c r="V10">
         <v>24855741222.2541</v>
       </c>
-      <c r="V10">
+      <c r="W10">
         <v>5.69914835773996</v>
       </c>
-      <c r="W10">
+      <c r="X10">
         <v>23.3500279730689</v>
       </c>
-      <c r="X10">
+      <c r="Y10">
         <v>12.65</v>
       </c>
     </row>
-    <row r="11" spans="1:24">
+    <row r="11" spans="1:25">
       <c r="A11" s="1">
         <v>1999</v>
       </c>
@@ -1134,49 +1167,52 @@
         <v>1730283000</v>
       </c>
       <c r="I11">
+        <v>283523000000</v>
+      </c>
+      <c r="J11">
         <v>-3.38545704063269</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>7705.54288252851</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>49.8</v>
       </c>
-      <c r="L11">
+      <c r="M11">
         <v>13.7232114149469</v>
       </c>
-      <c r="M11">
+      <c r="N11">
         <v>16.7436856974566</v>
       </c>
-      <c r="N11">
+      <c r="O11">
         <v>14.0111384261594</v>
       </c>
-      <c r="O11">
+      <c r="P11">
         <v>11.5555704475475</v>
       </c>
-      <c r="Q11">
+      <c r="R11">
         <v>17.2745311993124</v>
       </c>
-      <c r="R11">
+      <c r="S11">
         <v>-2.92441883021836</v>
       </c>
-      <c r="T11">
+      <c r="U11">
         <v>9.076124335591819</v>
       </c>
-      <c r="U11">
+      <c r="V11">
         <v>26350163486.3723</v>
       </c>
-      <c r="V11">
+      <c r="W11">
         <v>6.80464213303423</v>
       </c>
-      <c r="W11">
+      <c r="X11">
         <v>21.3827449624898</v>
       </c>
-      <c r="X11">
+      <c r="Y11">
         <v>14.05</v>
       </c>
     </row>
-    <row r="12" spans="1:24">
+    <row r="12" spans="1:25">
       <c r="A12" s="1">
         <v>2000</v>
       </c>
@@ -1202,52 +1238,55 @@
         <v>901028199.3378561</v>
       </c>
       <c r="I12">
+        <v>284203750000</v>
+      </c>
+      <c r="J12">
         <v>-0.78899893905691</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>7637.01489203628</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>51</v>
       </c>
-      <c r="L12">
+      <c r="M12">
         <v>13.7841913064131</v>
       </c>
-      <c r="M12">
+      <c r="N12">
         <v>16.8328883767368</v>
       </c>
-      <c r="N12">
+      <c r="O12">
         <v>14.1776102532074</v>
       </c>
-      <c r="O12">
+      <c r="P12">
         <v>11.6360695451767</v>
       </c>
-      <c r="Q12">
+      <c r="R12">
         <v>20.1040140301883</v>
       </c>
-      <c r="R12">
+      <c r="S12">
         <v>-2.77220128165093</v>
       </c>
-      <c r="S12">
+      <c r="T12">
         <v>0.0958238765597343</v>
       </c>
-      <c r="T12">
+      <c r="U12">
         <v>9.622603501889049</v>
       </c>
-      <c r="U12">
+      <c r="V12">
         <v>25152117244.4134</v>
       </c>
-      <c r="V12">
+      <c r="W12">
         <v>6.28322204626375</v>
       </c>
-      <c r="W12">
+      <c r="X12">
         <v>22.6224447777343</v>
       </c>
-      <c r="X12">
+      <c r="Y12">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:24">
+    <row r="13" spans="1:25">
       <c r="A13" s="1">
         <v>2001</v>
       </c>
@@ -1270,49 +1309,52 @@
         <v>160876687.495159</v>
       </c>
       <c r="I13">
+        <v>268696750000</v>
+      </c>
+      <c r="J13">
         <v>-4.40883968258557</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>7141.47507662826</v>
       </c>
-      <c r="K13">
+      <c r="L13">
         <v>53.3</v>
       </c>
-      <c r="L13">
+      <c r="M13">
         <v>14.1562743129569</v>
       </c>
-      <c r="M13">
+      <c r="N13">
         <v>16.9923529034125</v>
       </c>
-      <c r="N13">
+      <c r="O13">
         <v>13.7775019608536</v>
       </c>
-      <c r="O13">
+      <c r="P13">
         <v>10.2732473690136</v>
       </c>
-      <c r="Q13">
+      <c r="R13">
         <v>22.2743490173661</v>
       </c>
-      <c r="R13">
+      <c r="S13">
         <v>-3.31954145332982</v>
       </c>
-      <c r="T13">
+      <c r="U13">
         <v>9.324898793900561</v>
       </c>
-      <c r="U13">
+      <c r="V13">
         <v>14555552759.6102</v>
       </c>
-      <c r="V13">
+      <c r="W13">
         <v>4.29371406025342</v>
       </c>
-      <c r="W13">
+      <c r="X13">
         <v>21.8522554515453</v>
       </c>
-      <c r="X13">
+      <c r="Y13">
         <v>17.32</v>
       </c>
     </row>
-    <row r="14" spans="1:24">
+    <row r="14" spans="1:25">
       <c r="A14" s="1">
         <v>2002</v>
       </c>
@@ -1338,52 +1380,55 @@
         <v>-627140000</v>
       </c>
       <c r="I14">
+        <v>97724004251.8602</v>
+      </c>
+      <c r="J14">
         <v>-10.8944848285903</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>2569.69963519124</v>
       </c>
-      <c r="K14">
+      <c r="L14">
         <v>53.8</v>
       </c>
-      <c r="L14">
+      <c r="M14">
         <v>12.235247296692</v>
       </c>
-      <c r="M14">
+      <c r="N14">
         <v>19.6771706443151</v>
       </c>
-      <c r="N14">
+      <c r="O14">
         <v>14.0561136349095</v>
       </c>
-      <c r="O14">
+      <c r="P14">
         <v>13.370127359396</v>
       </c>
-      <c r="Q14">
+      <c r="R14">
         <v>34.2849338854665</v>
       </c>
-      <c r="R14">
+      <c r="S14">
         <v>-5.70628319150298</v>
       </c>
-      <c r="S14">
+      <c r="T14">
         <v>-0.776545405387878</v>
       </c>
-      <c r="T14">
+      <c r="U14">
         <v>9.81895834666325</v>
       </c>
-      <c r="U14">
+      <c r="V14">
         <v>10492424818.7375</v>
       </c>
-      <c r="V14">
+      <c r="W14">
         <v>5.27543170673442</v>
       </c>
-      <c r="W14">
+      <c r="X14">
         <v>41.7527243585642</v>
       </c>
-      <c r="X14">
+      <c r="Y14">
         <v>19.59</v>
       </c>
     </row>
-    <row r="15" spans="1:24">
+    <row r="15" spans="1:25">
       <c r="A15" s="1">
         <v>2003</v>
       </c>
@@ -1409,52 +1454,55 @@
         <v>773780000</v>
       </c>
       <c r="I15">
+        <v>127586973492.177</v>
+      </c>
+      <c r="J15">
         <v>8.837040795769241</v>
       </c>
-      <c r="J15">
+      <c r="K15">
         <v>3320.47775133903</v>
       </c>
-      <c r="K15">
+      <c r="L15">
         <v>51</v>
       </c>
-      <c r="L15">
+      <c r="M15">
         <v>11.4380567929249</v>
       </c>
-      <c r="M15">
+      <c r="N15">
         <v>19.8373029880995</v>
       </c>
-      <c r="N15">
+      <c r="O15">
         <v>17.1997019513553</v>
       </c>
-      <c r="O15">
+      <c r="P15">
         <v>14.7138051046861</v>
       </c>
-      <c r="Q15">
+      <c r="R15">
         <v>30.0083948621788</v>
       </c>
-      <c r="R15">
+      <c r="S15">
         <v>-2.82936804297577</v>
       </c>
-      <c r="S15">
+      <c r="T15">
         <v>-0.359838128089905</v>
       </c>
-      <c r="T15">
+      <c r="U15">
         <v>12.5187797002949</v>
       </c>
-      <c r="U15">
+      <c r="V15">
         <v>14157284136.3645</v>
       </c>
-      <c r="V15">
+      <c r="W15">
         <v>5.70013745215417</v>
       </c>
-      <c r="W15">
+      <c r="X15">
         <v>40.6447480311085</v>
       </c>
-      <c r="X15">
+      <c r="Y15">
         <v>15.36</v>
       </c>
     </row>
-    <row r="16" spans="1:24">
+    <row r="16" spans="1:25">
       <c r="A16" s="1">
         <v>2004</v>
       </c>
@@ -1480,52 +1528,55 @@
         <v>675990000</v>
       </c>
       <c r="I16">
+        <v>164657930452.787</v>
+      </c>
+      <c r="J16">
         <v>9.02957330068152</v>
       </c>
-      <c r="J16">
+      <c r="K16">
         <v>4242.02099089422</v>
       </c>
-      <c r="K16">
+      <c r="L16">
         <v>48.5</v>
       </c>
-      <c r="L16">
+      <c r="M16">
         <v>11.114636067696</v>
       </c>
-      <c r="M16">
+      <c r="N16">
         <v>16.8763416365527</v>
       </c>
-      <c r="N16">
+      <c r="O16">
         <v>16.7347777696665</v>
       </c>
-      <c r="O16">
+      <c r="P16">
         <v>16.8450266849578</v>
       </c>
-      <c r="Q16">
+      <c r="R16">
         <v>26.3142537893684</v>
       </c>
-      <c r="R16">
+      <c r="S16">
         <v>-0.425276316786125</v>
       </c>
-      <c r="S16">
+      <c r="T16">
         <v>-0.610934913158417</v>
       </c>
-      <c r="T16">
+      <c r="U16">
         <v>13.1007798994386</v>
       </c>
-      <c r="U16">
+      <c r="V16">
         <v>19659591803.9788</v>
       </c>
-      <c r="V16">
+      <c r="W16">
         <v>5.77837779911896</v>
       </c>
-      <c r="W16">
+      <c r="X16">
         <v>40.692646108947</v>
       </c>
-      <c r="X16">
+      <c r="Y16">
         <v>13.522</v>
       </c>
     </row>
-    <row r="17" spans="1:24">
+    <row r="17" spans="1:25">
       <c r="A17" s="1">
         <v>2005</v>
       </c>
@@ -1551,43 +1602,46 @@
         <v>1311060000</v>
       </c>
       <c r="I17">
+        <v>198737095012.282</v>
+      </c>
+      <c r="J17">
         <v>8.85165992013437</v>
       </c>
-      <c r="J17">
+      <c r="K17">
         <v>5067.65342293276</v>
       </c>
-      <c r="K17">
+      <c r="L17">
         <v>47.8</v>
       </c>
-      <c r="L17">
+      <c r="M17">
         <v>12.1418612359575</v>
       </c>
-      <c r="N17">
+      <c r="O17">
         <v>16.6216575161027</v>
       </c>
-      <c r="O17">
+      <c r="P17">
         <v>17.3053942367662</v>
       </c>
-      <c r="S17">
+      <c r="T17">
         <v>-0.0417749434709549</v>
       </c>
-      <c r="T17">
+      <c r="U17">
         <v>13.1031756459852</v>
       </c>
-      <c r="U17">
+      <c r="V17">
         <v>28081718501.5579</v>
       </c>
-      <c r="V17">
+      <c r="W17">
         <v>7.26029776298214</v>
       </c>
-      <c r="W17">
+      <c r="X17">
         <v>40.5512709706238</v>
       </c>
-      <c r="X17">
+      <c r="Y17">
         <v>11.506</v>
       </c>
     </row>
-    <row r="18" spans="1:24">
+    <row r="18" spans="1:25">
       <c r="A18" s="1">
         <v>2006</v>
       </c>
@@ -1613,43 +1667,46 @@
         <v>2438720720.56097</v>
       </c>
       <c r="I18">
+        <v>232557260817.308</v>
+      </c>
+      <c r="J18">
         <v>8.047151500430269</v>
       </c>
-      <c r="J18">
+      <c r="K18">
         <v>5869.38028970204</v>
       </c>
-      <c r="K18">
+      <c r="L18">
         <v>46.4</v>
       </c>
-      <c r="L18">
+      <c r="M18">
         <v>12.4294153726307</v>
       </c>
-      <c r="N18">
+      <c r="O18">
         <v>17.2017551603052</v>
       </c>
-      <c r="O18">
+      <c r="P18">
         <v>17.4067852681036</v>
       </c>
-      <c r="S18">
+      <c r="T18">
         <v>0.00196776282973588</v>
       </c>
-      <c r="T18">
+      <c r="U18">
         <v>12.8788866954319</v>
       </c>
-      <c r="U18">
+      <c r="V18">
         <v>32022297112.9806</v>
       </c>
-      <c r="V18">
+      <c r="W18">
         <v>7.02897239370493</v>
       </c>
-      <c r="W18">
+      <c r="X18">
         <v>40.4334798719151</v>
       </c>
-      <c r="X18">
+      <c r="Y18">
         <v>10.078</v>
       </c>
     </row>
-    <row r="19" spans="1:24">
+    <row r="19" spans="1:25">
       <c r="A19" s="1">
         <v>2007</v>
       </c>
@@ -1675,43 +1732,46 @@
         <v>1504232961.34457</v>
       </c>
       <c r="I19">
+        <v>287530508430.568</v>
+      </c>
+      <c r="J19">
         <v>9.00765087504757</v>
       </c>
-      <c r="J19">
+      <c r="K19">
         <v>7185.25155147027</v>
       </c>
-      <c r="K19">
+      <c r="L19">
         <v>46.3</v>
       </c>
-      <c r="L19">
+      <c r="M19">
         <v>12.9893238963619</v>
       </c>
-      <c r="N19">
+      <c r="O19">
         <v>17.9300729987004</v>
       </c>
-      <c r="O19">
+      <c r="P19">
         <v>18.2824203070644</v>
       </c>
-      <c r="S19">
+      <c r="T19">
         <v>0.0977966338396072</v>
       </c>
-      <c r="T19">
+      <c r="U19">
         <v>12.4482684483004</v>
       </c>
-      <c r="U19">
+      <c r="V19">
         <v>46149456855.7802</v>
       </c>
-      <c r="V19">
+      <c r="W19">
         <v>8.171534286186461</v>
       </c>
-      <c r="W19">
+      <c r="X19">
         <v>40.945170618571</v>
       </c>
-      <c r="X19">
+      <c r="Y19">
         <v>8.470000000000001</v>
       </c>
     </row>
-    <row r="20" spans="1:24">
+    <row r="20" spans="1:25">
       <c r="A20" s="1">
         <v>2008</v>
       </c>
@@ -1737,43 +1797,46 @@
         <v>1390934588.87756</v>
       </c>
       <c r="I20">
+        <v>361558037110.419</v>
+      </c>
+      <c r="J20">
         <v>4.05723310346406</v>
       </c>
-      <c r="J20">
+      <c r="K20">
         <v>8944.110265735701</v>
       </c>
-      <c r="K20">
+      <c r="L20">
         <v>45</v>
       </c>
-      <c r="L20">
+      <c r="M20">
         <v>13.6335132595631</v>
       </c>
-      <c r="N20">
+      <c r="O20">
         <v>18.9717341522181</v>
       </c>
-      <c r="O20">
+      <c r="P20">
         <v>18.341772996414</v>
       </c>
-      <c r="S20">
+      <c r="T20">
         <v>-0.0877556875348091</v>
       </c>
-      <c r="T20">
+      <c r="U20">
         <v>13.3178463574032</v>
       </c>
-      <c r="U20">
+      <c r="V20">
         <v>46385380206.9801</v>
       </c>
-      <c r="V20">
+      <c r="W20">
         <v>6.71425831138327</v>
       </c>
-      <c r="W20">
+      <c r="X20">
         <v>40.4026733790382</v>
       </c>
-      <c r="X20">
+      <c r="Y20">
         <v>7.837</v>
       </c>
     </row>
-    <row r="21" spans="1:24">
+    <row r="21" spans="1:25">
       <c r="A21" s="1">
         <v>2009</v>
       </c>
@@ -1799,43 +1862,46 @@
         <v>711546403.745669</v>
       </c>
       <c r="I21">
+        <v>332976484577.619</v>
+      </c>
+      <c r="J21">
         <v>-5.91852507634947</v>
       </c>
-      <c r="J21">
+      <c r="K21">
         <v>8150.23527028221</v>
       </c>
-      <c r="K21">
+      <c r="L21">
         <v>43.8</v>
       </c>
-      <c r="L21">
+      <c r="M21">
         <v>15.903896746884</v>
       </c>
-      <c r="N21">
+      <c r="O21">
         <v>20.1360210279783</v>
       </c>
-      <c r="O21">
+      <c r="P21">
         <v>14.4961418494061</v>
       </c>
-      <c r="S21">
+      <c r="T21">
         <v>-0.234854578971863</v>
       </c>
-      <c r="T21">
+      <c r="U21">
         <v>12.3830415594157</v>
       </c>
-      <c r="U21">
+      <c r="V21">
         <v>48006988635.3253</v>
       </c>
-      <c r="V21">
+      <c r="W21">
         <v>9.067499928752429</v>
       </c>
-      <c r="W21">
+      <c r="X21">
         <v>34.0571269054879</v>
       </c>
-      <c r="X21">
+      <c r="Y21">
         <v>8.645</v>
       </c>
     </row>
-    <row r="22" spans="1:24">
+    <row r="22" spans="1:25">
       <c r="A22" s="1">
         <v>2010</v>
       </c>
@@ -1861,43 +1927,46 @@
         <v>964760680.391807</v>
       </c>
       <c r="I22">
+        <v>423627422092.49</v>
+      </c>
+      <c r="J22">
         <v>10.1253981561002</v>
       </c>
-      <c r="J22">
+      <c r="K22">
         <v>10260.1313108254</v>
       </c>
-      <c r="K22">
+      <c r="L22">
         <v>43.7</v>
       </c>
-      <c r="L22">
+      <c r="M22">
         <v>15.1637178886417</v>
       </c>
-      <c r="N22">
+      <c r="O22">
         <v>21.2413164267537</v>
       </c>
-      <c r="O22">
+      <c r="P22">
         <v>16.0371898581987</v>
       </c>
-      <c r="S22">
+      <c r="T22">
         <v>-0.0847978666424751</v>
       </c>
-      <c r="T22">
+      <c r="U22">
         <v>12.8530426903255</v>
       </c>
-      <c r="U22">
+      <c r="V22">
         <v>52207549724.0928</v>
       </c>
-      <c r="V22">
+      <c r="W22">
         <v>7.27697103967374</v>
       </c>
-      <c r="W22">
+      <c r="X22">
         <v>34.9710132635696</v>
       </c>
-      <c r="X22">
+      <c r="Y22">
         <v>7.714</v>
       </c>
     </row>
-    <row r="23" spans="1:24">
+    <row r="23" spans="1:25">
       <c r="A23" s="1">
         <v>2011</v>
       </c>
@@ -1923,43 +1992,46 @@
         <v>1488000000</v>
       </c>
       <c r="I23">
+        <v>530158122010.442</v>
+      </c>
+      <c r="J23">
         <v>6.00395169280579</v>
       </c>
-      <c r="J23">
+      <c r="K23">
         <v>12704.2831819684</v>
       </c>
-      <c r="K23">
+      <c r="L23">
         <v>42.7</v>
       </c>
-      <c r="L23">
+      <c r="M23">
         <v>15.6889565165983</v>
       </c>
-      <c r="N23">
+      <c r="O23">
         <v>20.196408074281</v>
       </c>
-      <c r="O23">
+      <c r="P23">
         <v>16.7569458546489</v>
       </c>
-      <c r="S23">
+      <c r="T23">
         <v>0.158993661403656</v>
       </c>
-      <c r="T23">
+      <c r="U23">
         <v>12.6636277012315</v>
       </c>
-      <c r="U23">
+      <c r="V23">
         <v>46265800525.8807</v>
       </c>
-      <c r="V23">
+      <c r="W23">
         <v>5.20195157798821</v>
       </c>
-      <c r="W23">
+      <c r="X23">
         <v>35.2061549999644</v>
       </c>
-      <c r="X23">
+      <c r="Y23">
         <v>7.18</v>
       </c>
     </row>
-    <row r="24" spans="1:24">
+    <row r="24" spans="1:25">
       <c r="A24" s="1">
         <v>2012</v>
       </c>
@@ -1985,43 +2057,46 @@
         <v>1054849578.05632</v>
       </c>
       <c r="I24">
+        <v>545982375701.128</v>
+      </c>
+      <c r="J24">
         <v>-1.0264204544321</v>
       </c>
-      <c r="J24">
+      <c r="K24">
         <v>12949.717486654</v>
       </c>
-      <c r="K24">
+      <c r="L24">
         <v>41.4</v>
       </c>
-      <c r="L24">
+      <c r="M24">
         <v>16.6454378106252</v>
       </c>
-      <c r="N24">
+      <c r="O24">
         <v>21.182234604867</v>
       </c>
-      <c r="O24">
+      <c r="P24">
         <v>14.2886829096862</v>
       </c>
-      <c r="S24">
+      <c r="T24">
         <v>0.103040546178818</v>
       </c>
-      <c r="T24">
+      <c r="U24">
         <v>12.9528415127413</v>
       </c>
-      <c r="U24">
+      <c r="V24">
         <v>43223270863.843</v>
       </c>
-      <c r="V24">
+      <c r="W24">
         <v>5.21829041219894</v>
       </c>
-      <c r="W24">
+      <c r="X24">
         <v>30.5265423717108</v>
       </c>
-      <c r="X24">
+      <c r="Y24">
         <v>7.217</v>
       </c>
     </row>
-    <row r="25" spans="1:24">
+    <row r="25" spans="1:25">
       <c r="A25" s="1">
         <v>2013</v>
       </c>
@@ -2047,43 +2122,46 @@
         <v>889972858.727091</v>
       </c>
       <c r="I25">
+        <v>552025140252.246</v>
+      </c>
+      <c r="J25">
         <v>2.40532378079436</v>
       </c>
-      <c r="J25">
+      <c r="K25">
         <v>12963.675773326</v>
       </c>
-      <c r="K25">
+      <c r="L25">
         <v>41.1</v>
       </c>
-      <c r="L25">
+      <c r="M25">
         <v>16.8062377968797</v>
       </c>
-      <c r="N25">
+      <c r="O25">
         <v>21.5652829643596</v>
       </c>
-      <c r="O25">
+      <c r="P25">
         <v>14.7167556136651</v>
       </c>
-      <c r="S25">
+      <c r="T25">
         <v>0.0653142631053925</v>
       </c>
-      <c r="T25">
+      <c r="U25">
         <v>12.4529027558077</v>
       </c>
-      <c r="U25">
+      <c r="V25">
         <v>30533919650.6264</v>
       </c>
-      <c r="V25">
+      <c r="W25">
         <v>3.46015205462158</v>
       </c>
-      <c r="W25">
+      <c r="X25">
         <v>29.3339290021037</v>
       </c>
-      <c r="X25">
+      <c r="Y25">
         <v>7.1</v>
       </c>
     </row>
-    <row r="26" spans="1:24">
+    <row r="26" spans="1:25">
       <c r="A26" s="1">
         <v>2014</v>
       </c>
@@ -2109,52 +2187,55 @@
         <v>1920541433.10504</v>
       </c>
       <c r="I26">
+        <v>526319673731.638</v>
+      </c>
+      <c r="J26">
         <v>-2.51261532081394</v>
       </c>
-      <c r="J26">
+      <c r="K26">
         <v>12233.1444119186</v>
       </c>
-      <c r="K26">
+      <c r="L26">
         <v>41.8</v>
       </c>
-      <c r="L26">
+      <c r="M26">
         <v>16.9498757371062</v>
       </c>
-      <c r="M26">
+      <c r="N26">
         <v>24.5697808575806</v>
       </c>
-      <c r="N26">
+      <c r="O26">
         <v>22.3322943705014</v>
       </c>
-      <c r="O26">
+      <c r="P26">
         <v>14.0013150558519</v>
       </c>
-      <c r="Q26">
+      <c r="R26">
         <v>7.75788916526639</v>
       </c>
-      <c r="R26">
+      <c r="S26">
         <v>-2.90614606577065</v>
       </c>
-      <c r="S26">
+      <c r="T26">
         <v>-0.00512187136337161</v>
       </c>
-      <c r="T26">
+      <c r="U26">
         <v>12.6109666067191</v>
       </c>
-      <c r="U26">
+      <c r="V26">
         <v>31410813269.5239</v>
       </c>
-      <c r="V26">
+      <c r="W26">
         <v>3.96299919336678</v>
       </c>
-      <c r="W26">
+      <c r="X26">
         <v>28.4067936452275</v>
       </c>
-      <c r="X26">
+      <c r="Y26">
         <v>7.268</v>
       </c>
     </row>
-    <row r="27" spans="1:24">
+    <row r="27" spans="1:25">
       <c r="A27" s="1">
         <v>2015</v>
       </c>
@@ -2180,49 +2261,52 @@
         <v>875233227.3542579</v>
       </c>
       <c r="I27">
+        <v>594749285413.212</v>
+      </c>
+      <c r="J27">
         <v>2.73115982828944</v>
       </c>
-      <c r="J27">
+      <c r="K27">
         <v>13679.6264980954</v>
       </c>
-      <c r="L27">
+      <c r="M27">
         <v>18.098379759087</v>
       </c>
-      <c r="M27">
+      <c r="N27">
         <v>25.0083932347048</v>
       </c>
-      <c r="N27">
+      <c r="O27">
         <v>22.1490803040164</v>
       </c>
-      <c r="O27">
+      <c r="P27">
         <v>11.7805740385254</v>
       </c>
-      <c r="Q27">
+      <c r="R27">
         <v>7.37421073749561</v>
       </c>
-      <c r="R27">
+      <c r="S27">
         <v>-3.39011034719535</v>
       </c>
-      <c r="S27">
+      <c r="T27">
         <v>0.00876413471996784</v>
       </c>
-      <c r="T27">
+      <c r="U27">
         <v>12.3365069418291</v>
       </c>
-      <c r="U27">
+      <c r="V27">
         <v>25520565580.4894</v>
       </c>
-      <c r="V27">
+      <c r="W27">
         <v>3.36214425707702</v>
       </c>
-      <c r="W27">
+      <c r="X27">
         <v>22.4862260889792</v>
       </c>
-      <c r="X27">
+      <c r="Y27">
         <v>7.579</v>
       </c>
     </row>
-    <row r="28" spans="1:24">
+    <row r="28" spans="1:25">
       <c r="A28" s="1">
         <v>2016</v>
       </c>
@@ -2248,52 +2332,55 @@
         <v>1786530934.74804</v>
       </c>
       <c r="I28">
+        <v>557532320662.955</v>
+      </c>
+      <c r="J28">
         <v>-2.08032784377811</v>
       </c>
-      <c r="J28">
+      <c r="K28">
         <v>12699.9623137756</v>
       </c>
-      <c r="K28">
+      <c r="L28">
         <v>42.3</v>
       </c>
-      <c r="L28">
+      <c r="M28">
         <v>17.6545781863509</v>
       </c>
-      <c r="M28">
+      <c r="N28">
         <v>26.1799164832469</v>
       </c>
-      <c r="N28">
+      <c r="O28">
         <v>21.2567013071388</v>
       </c>
-      <c r="O28">
+      <c r="P28">
         <v>13.5667926798789</v>
       </c>
-      <c r="Q28">
+      <c r="R28">
         <v>11.3900941602608</v>
       </c>
-      <c r="R28">
+      <c r="S28">
         <v>-5.33377782706346</v>
       </c>
-      <c r="S28">
+      <c r="T28">
         <v>0.197749897837639</v>
       </c>
-      <c r="T28">
+      <c r="U28">
         <v>12.0972836411962</v>
       </c>
-      <c r="U28">
+      <c r="V28">
         <v>38414518491.6132</v>
       </c>
-      <c r="V28">
+      <c r="W28">
         <v>5.09719624487539</v>
       </c>
-      <c r="W28">
+      <c r="X28">
         <v>26.0938878488799</v>
       </c>
-      <c r="X28">
+      <c r="Y28">
         <v>8.085000000000001</v>
       </c>
     </row>
-    <row r="29" spans="1:24">
+    <row r="29" spans="1:25">
       <c r="A29" s="1">
         <v>2017</v>
       </c>
@@ -2319,52 +2406,55 @@
         <v>1155630218.02452</v>
       </c>
       <c r="I29">
+        <v>643628393281.364</v>
+      </c>
+      <c r="J29">
         <v>2.81850297775918</v>
       </c>
-      <c r="J29">
+      <c r="K29">
         <v>14532.5009308511</v>
       </c>
-      <c r="K29">
+      <c r="L29">
         <v>41.4</v>
       </c>
-      <c r="L29">
+      <c r="M29">
         <v>17.6968939223042</v>
       </c>
-      <c r="M29">
+      <c r="N29">
         <v>24.2825320419979</v>
       </c>
-      <c r="N29">
+      <c r="O29">
         <v>19.3371239744582</v>
       </c>
-      <c r="O29">
+      <c r="P29">
         <v>13.9693177780045</v>
       </c>
-      <c r="Q29">
+      <c r="R29">
         <v>9.419814018022439</v>
       </c>
-      <c r="R29">
+      <c r="S29">
         <v>-5.51824569508007</v>
       </c>
-      <c r="S29">
+      <c r="T29">
         <v>0.162542164325714</v>
       </c>
-      <c r="T29">
+      <c r="U29">
         <v>10.939623860491</v>
       </c>
-      <c r="U29">
+      <c r="V29">
         <v>55314409205.2189</v>
       </c>
-      <c r="V29">
+      <c r="W29">
         <v>6.05038766582561</v>
       </c>
-      <c r="W29">
+      <c r="X29">
         <v>25.2896011376779</v>
       </c>
-      <c r="X29">
+      <c r="Y29">
         <v>8.347</v>
       </c>
     </row>
-    <row r="30" spans="1:24">
+    <row r="30" spans="1:25">
       <c r="A30" s="1">
         <v>2018</v>
       </c>
@@ -2390,55 +2480,58 @@
         <v>1725981572.7057</v>
       </c>
       <c r="I30">
+        <v>524819892360.176</v>
+      </c>
+      <c r="J30">
         <v>-2.61739646282038</v>
       </c>
-      <c r="J30">
+      <c r="K30">
         <v>11752.7998922979</v>
       </c>
-      <c r="K30">
+      <c r="L30">
         <v>41.7</v>
       </c>
-      <c r="L30">
+      <c r="M30">
         <v>15.8050971558947</v>
       </c>
-      <c r="M30">
+      <c r="N30">
         <v>22.6709430512171</v>
       </c>
-      <c r="N30">
+      <c r="O30">
         <v>17.7024488717292</v>
       </c>
-      <c r="O30">
+      <c r="P30">
         <v>16.3258502050892</v>
       </c>
-      <c r="P30">
+      <c r="Q30">
         <v>34.2772237131003</v>
       </c>
-      <c r="Q30">
+      <c r="R30">
         <v>12.8793045637226</v>
       </c>
-      <c r="R30">
+      <c r="S30">
         <v>-5.33635226717988</v>
       </c>
-      <c r="S30">
+      <c r="T30">
         <v>0.00690981233492494</v>
       </c>
-      <c r="T30">
+      <c r="U30">
         <v>9.79144712037089</v>
       </c>
-      <c r="U30">
+      <c r="V30">
         <v>66221501691.4418</v>
       </c>
-      <c r="V30">
+      <c r="W30">
         <v>7.11111211150086</v>
       </c>
-      <c r="W30">
+      <c r="X30">
         <v>30.7625359549926</v>
       </c>
-      <c r="X30">
+      <c r="Y30">
         <v>9.220000000000001</v>
       </c>
     </row>
-    <row r="31" spans="1:24">
+    <row r="31" spans="1:25">
       <c r="A31" s="1">
         <v>2019</v>
       </c>
@@ -2464,55 +2557,58 @@
         <v>1522728151.79532</v>
       </c>
       <c r="I31">
+        <v>447754683615.225</v>
+      </c>
+      <c r="J31">
         <v>-2.00086100285785</v>
       </c>
-      <c r="J31">
+      <c r="K31">
         <v>9955.97478680428</v>
       </c>
-      <c r="K31">
+      <c r="L31">
         <v>43.3</v>
       </c>
-      <c r="L31">
+      <c r="M31">
         <v>16.4432415862976</v>
       </c>
-      <c r="M31">
+      <c r="N31">
         <v>22.0364845686943</v>
       </c>
-      <c r="N31">
+      <c r="O31">
         <v>17.7888990504455</v>
       </c>
-      <c r="O31">
+      <c r="P31">
         <v>14.7057366680037</v>
       </c>
-      <c r="P31">
+      <c r="Q31">
         <v>53.5483043492339</v>
       </c>
-      <c r="Q31">
+      <c r="R31">
         <v>15.7967986276777</v>
       </c>
-      <c r="R31">
+      <c r="S31">
         <v>-4.92889704924096</v>
       </c>
-      <c r="S31">
+      <c r="T31">
         <v>-0.0978230908513069</v>
       </c>
-      <c r="T31">
+      <c r="U31">
         <v>10.3919973375121</v>
       </c>
-      <c r="U31">
+      <c r="V31">
         <v>44880566052.3703</v>
       </c>
-      <c r="V31">
+      <c r="W31">
         <v>5.94220121846315</v>
       </c>
-      <c r="W31">
+      <c r="X31">
         <v>32.6306150458499</v>
       </c>
-      <c r="X31">
+      <c r="Y31">
         <v>9.843</v>
       </c>
     </row>
-    <row r="32" spans="1:24">
+    <row r="32" spans="1:25">
       <c r="A32" s="1">
         <v>2020</v>
       </c>
@@ -2538,55 +2634,58 @@
         <v>1177176908.60545</v>
       </c>
       <c r="I32">
+        <v>385740508436.965</v>
+      </c>
+      <c r="J32">
         <v>-9.900484813646401</v>
       </c>
-      <c r="J32">
+      <c r="K32">
         <v>8535.59938004389</v>
       </c>
-      <c r="K32">
+      <c r="L32">
         <v>42.7</v>
       </c>
-      <c r="L32">
+      <c r="M32">
         <v>16.8730073837365</v>
       </c>
-      <c r="M32">
+      <c r="N32">
         <v>25.8405452538391</v>
       </c>
-      <c r="N32">
+      <c r="O32">
         <v>17.4777322783093</v>
       </c>
-      <c r="O32">
+      <c r="P32">
         <v>13.5982843701675</v>
       </c>
-      <c r="P32">
+      <c r="Q32">
         <v>42.0150947376509</v>
       </c>
-      <c r="Q32">
+      <c r="R32">
         <v>7.50264305918987</v>
       </c>
-      <c r="R32">
+      <c r="S32">
         <v>-8.6954919523039</v>
       </c>
-      <c r="S32">
+      <c r="T32">
         <v>-0.0719974040985107</v>
       </c>
-      <c r="T32">
+      <c r="U32">
         <v>10.70812114449</v>
       </c>
-      <c r="U32">
+      <c r="V32">
         <v>39403734630.1228</v>
       </c>
-      <c r="V32">
+      <c r="W32">
         <v>7.09405401009515</v>
       </c>
-      <c r="W32">
+      <c r="X32">
         <v>30.203698807416</v>
       </c>
-      <c r="X32">
+      <c r="Y32">
         <v>11.461</v>
       </c>
     </row>
-    <row r="33" spans="1:24">
+    <row r="33" spans="1:25">
       <c r="A33" s="1">
         <v>2021</v>
       </c>
@@ -2612,55 +2711,58 @@
         <v>1543861737.75886</v>
       </c>
       <c r="I33">
+        <v>486564085480.036</v>
+      </c>
+      <c r="J33">
         <v>10.4418119882506</v>
       </c>
-      <c r="J33">
+      <c r="K33">
         <v>10738.0179223384</v>
       </c>
-      <c r="K33">
+      <c r="L33">
         <v>42.4</v>
       </c>
-      <c r="L33">
+      <c r="M33">
         <v>15.9158179423023</v>
       </c>
-      <c r="M33">
+      <c r="N33">
         <v>22.8967903877811</v>
       </c>
-      <c r="N33">
+      <c r="O33">
         <v>18.0764989044589</v>
       </c>
-      <c r="O33">
+      <c r="P33">
         <v>15.0119803984295</v>
       </c>
-      <c r="P33">
+      <c r="Q33">
         <v>48.4093786255199</v>
       </c>
-      <c r="Q33">
+      <c r="R33">
         <v>6.52367466313931</v>
       </c>
-      <c r="R33">
+      <c r="S33">
         <v>-4.37239542495983</v>
       </c>
-      <c r="S33">
+      <c r="T33">
         <v>0.000530058634467423</v>
       </c>
-      <c r="T33">
+      <c r="U33">
         <v>11.3410740330927</v>
       </c>
-      <c r="U33">
+      <c r="V33">
         <v>39653498610.7828</v>
       </c>
-      <c r="V33">
+      <c r="W33">
         <v>5.6049034262494</v>
       </c>
-      <c r="W33">
+      <c r="X33">
         <v>33.078689567466</v>
       </c>
-      <c r="X33">
+      <c r="Y33">
         <v>8.736000000000001</v>
       </c>
     </row>
-    <row r="34" spans="1:24">
+    <row r="34" spans="1:25">
       <c r="A34" s="1">
         <v>2022</v>
       </c>
@@ -2686,55 +2788,58 @@
         <v>2089836583.05669</v>
       </c>
       <c r="I34">
+        <v>632790070063.124</v>
+      </c>
+      <c r="J34">
         <v>5.26987967384072</v>
       </c>
-      <c r="J34">
+      <c r="K34">
         <v>13935.6811110049</v>
       </c>
-      <c r="K34">
+      <c r="L34">
         <v>40.7</v>
       </c>
-      <c r="L34">
+      <c r="M34">
         <v>15.8356571842994</v>
       </c>
-      <c r="M34">
+      <c r="N34">
         <v>21.9068187207194</v>
       </c>
-      <c r="N34">
+      <c r="O34">
         <v>17.9272315382489</v>
       </c>
-      <c r="O34">
+      <c r="P34">
         <v>15.2996935612041</v>
       </c>
-      <c r="P34">
+      <c r="Q34">
         <v>72.430757531824</v>
       </c>
-      <c r="Q34">
+      <c r="R34">
         <v>7.76084028840006</v>
       </c>
-      <c r="R34">
+      <c r="S34">
         <v>-4.43550847563459</v>
       </c>
-      <c r="S34">
+      <c r="T34">
         <v>-0.0985943302512169</v>
       </c>
-      <c r="T34">
+      <c r="U34">
         <v>11.0858180930687</v>
       </c>
-      <c r="U34">
+      <c r="V34">
         <v>44795335171.5152</v>
       </c>
-      <c r="V34">
+      <c r="W34">
         <v>4.75930856415363</v>
       </c>
-      <c r="W34">
+      <c r="X34">
         <v>31.5477080051071</v>
       </c>
-      <c r="X34">
+      <c r="Y34">
         <v>6.805</v>
       </c>
     </row>
-    <row r="35" spans="1:24">
+    <row r="35" spans="1:25">
       <c r="A35" s="1">
         <v>2023</v>
       </c>
@@ -2760,55 +2865,58 @@
         <v>3023263070.30906</v>
       </c>
       <c r="I35">
+        <v>646075277525.125</v>
+      </c>
+      <c r="J35">
         <v>-1.61100162090189</v>
       </c>
-      <c r="J35">
+      <c r="K35">
         <v>14187.4827252965</v>
       </c>
-      <c r="K35">
+      <c r="L35">
         <v>42.4</v>
       </c>
-      <c r="L35">
+      <c r="M35">
         <v>16.3874689950096</v>
       </c>
-      <c r="M35">
+      <c r="N35">
         <v>21.1189070510753</v>
       </c>
-      <c r="N35">
+      <c r="O35">
         <v>17.8684969726739</v>
       </c>
-      <c r="O35">
+      <c r="P35">
         <v>13.8912663507893</v>
       </c>
-      <c r="P35">
+      <c r="Q35">
         <v>133.488935594175</v>
       </c>
-      <c r="Q35">
+      <c r="R35">
         <v>7.28994415748098</v>
       </c>
-      <c r="R35">
+      <c r="S35">
         <v>-3.61371624476762</v>
       </c>
-      <c r="S35">
+      <c r="T35">
         <v>-0.127517908811569</v>
       </c>
-      <c r="T35">
+      <c r="U35">
         <v>9.98093648141313</v>
       </c>
-      <c r="U35">
+      <c r="V35">
         <v>23080560550.2946</v>
       </c>
-      <c r="V35">
+      <c r="W35">
         <v>2.45755251575411</v>
       </c>
-      <c r="W35">
+      <c r="X35">
         <v>26.6405121334437</v>
       </c>
-      <c r="X35">
+      <c r="Y35">
         <v>6.139</v>
       </c>
     </row>
-    <row r="36" spans="1:24">
+    <row r="36" spans="1:25">
       <c r="A36" s="1">
         <v>2024</v>
       </c>
@@ -2825,33 +2933,36 @@
         <v>2756722688.00138</v>
       </c>
       <c r="I36">
+        <v>633266692533.689</v>
+      </c>
+      <c r="J36">
         <v>-1.71910514722377</v>
       </c>
-      <c r="J36">
+      <c r="K36">
         <v>13858.2039802008</v>
       </c>
-      <c r="K36">
+      <c r="L36">
         <v>42.4</v>
       </c>
-      <c r="L36">
+      <c r="M36">
         <v>15.0308136208788</v>
       </c>
-      <c r="O36">
+      <c r="P36">
         <v>12.8251676959106</v>
       </c>
-      <c r="P36">
+      <c r="Q36">
         <v>219.883929014578</v>
       </c>
-      <c r="U36">
+      <c r="V36">
         <v>29559610350.7831</v>
       </c>
-      <c r="V36">
+      <c r="W36">
         <v>3.55326074207238</v>
       </c>
-      <c r="W36">
+      <c r="X36">
         <v>28.1594014348782</v>
       </c>
-      <c r="X36">
+      <c r="Y36">
         <v>7.876</v>
       </c>
     </row>

</xml_diff>